<commit_message>
fix bug import category
</commit_message>
<xml_diff>
--- a/public/CategoryData/category.xlsx
+++ b/public/CategoryData/category.xlsx
@@ -24,10 +24,10 @@
     <t>ID</t>
   </si>
   <si>
-    <t>Test Category</t>
+    <t>Nama Category</t>
   </si>
   <si>
-    <t>Nama Category</t>
+    <t>Test Category 1000</t>
   </si>
 </sst>
 </file>
@@ -389,7 +389,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
@@ -397,7 +397,7 @@
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">

</xml_diff>